<commit_message>
Populate university short names, resolve duplicate keys, and update aggregates
</commit_message>
<xml_diff>
--- a/Источники/файлы данных/Gr_prog.xlsx
+++ b/Источники/файлы данных/Gr_prog.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gr_pr" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -522,7 +522,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -576,7 +576,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>121</v>
       </c>
       <c r="B3" t="n">
         <v>1</v>
@@ -586,7 +586,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГХТхнУ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Сев(Аркт)ФУ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГВМетИ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КубГТхнУ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БелГТхнУ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтФУ</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГВМетИ</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтФУ</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГУ</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГТУ</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтФУ</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КрГТУ</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2946,7 +2946,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВолгГУ</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3522,7 +3522,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГГУ</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ЮЗГУ</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3834,7 +3834,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГВМетИ</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БрянГИТА</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -4142,7 +4142,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГГУ</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ЛипГТУ</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГТУ</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БрянГТУ</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БрянГТУ</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтГТУ</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КубГТхнУ</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВФУ</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КрГАСА</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КнАГТУ</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтФУ</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -5410,7 +5410,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГУПищП</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БашГУ</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -5758,7 +5758,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВФУ</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КострГТУ</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -5950,7 +5950,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ГУЦМиЗ</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -6206,7 +6206,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГУ</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -6270,7 +6270,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ЮЗГУ</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -6394,7 +6394,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -6586,7 +6586,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -6970,7 +6970,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВГТУ</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -7162,7 +7162,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БрянГИТА</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -7226,7 +7226,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -7354,7 +7354,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КузГТУ</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -7418,7 +7418,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КузГТУ</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -7482,7 +7482,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГВМетИ</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -7610,7 +7610,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГГУ</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГУ</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -7802,7 +7802,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтФУ</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -7866,7 +7866,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -7930,7 +7930,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КрГТУ</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВолгГТУ</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВГТУ</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -8122,7 +8122,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДагГУ</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -8250,7 +8250,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтГТУ</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -8378,7 +8378,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -8442,7 +8442,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтГТУ</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -8506,7 +8506,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГУ</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -8570,7 +8570,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВологГТУ</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -8634,7 +8634,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -8694,7 +8694,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КоврГТА</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -8812,7 +8812,7 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>21</v>
+        <v>471</v>
       </c>
       <c r="B134" t="n">
         <v>7</v>
@@ -8822,7 +8822,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -8886,7 +8886,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -8950,7 +8950,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГГУ</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -9078,7 +9078,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -9206,7 +9206,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГГУ</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВятГУ</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -9398,7 +9398,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -9462,7 +9462,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -9654,7 +9654,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -9718,7 +9718,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГЭУ</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГЭУ</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -9842,7 +9842,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -9902,7 +9902,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДагГТУ</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -9966,7 +9966,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДагГТУ</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -10030,7 +10030,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГЭУ</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -10094,7 +10094,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -10222,7 +10222,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГУНГ</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -10286,7 +10286,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -10350,7 +10350,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -10414,7 +10414,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВолгГУ</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -10478,7 +10478,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -10598,7 +10598,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГЭУ</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -10662,7 +10662,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -10790,7 +10790,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -10854,7 +10854,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -10914,7 +10914,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВГТУ</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -10978,7 +10978,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -11042,7 +11042,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -11106,7 +11106,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КургГУ</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -11170,7 +11170,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -11234,7 +11234,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БайГУЭП</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -11298,7 +11298,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГХТхнУ</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -11426,7 +11426,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -11490,7 +11490,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КубГУ</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -11554,7 +11554,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВологГТУ</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВФУ</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -11746,7 +11746,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МарГУ</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -11810,7 +11810,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -11874,7 +11874,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -12002,7 +12002,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
@@ -12066,7 +12066,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -12130,7 +12130,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -12194,7 +12194,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАМИ</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -12258,7 +12258,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -12322,7 +12322,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГУ</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -12386,7 +12386,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -12450,7 +12450,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -12514,7 +12514,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -12578,7 +12578,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГХТхнУ</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -12642,7 +12642,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -12706,7 +12706,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВГТУ</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -12770,7 +12770,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИжГТУ</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
@@ -12834,7 +12834,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -12894,7 +12894,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВФУ</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
@@ -12958,7 +12958,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -13022,7 +13022,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -13082,7 +13082,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КургГУ</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -13274,7 +13274,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -13338,7 +13338,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -13402,7 +13402,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -13466,7 +13466,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -13530,7 +13530,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГУП</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -13590,7 +13590,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КБГУ</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
@@ -13654,7 +13654,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -13718,7 +13718,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтГТУ</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
@@ -13782,7 +13782,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВФУ</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -13846,7 +13846,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -13910,7 +13910,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
@@ -13974,7 +13974,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -14038,7 +14038,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
@@ -14102,7 +14102,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГУ</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -14166,7 +14166,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГТУ</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
@@ -14230,7 +14230,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КубГУ</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтГТУ</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -14358,7 +14358,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -14422,7 +14422,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ЛипГТУ</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -14486,7 +14486,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
@@ -14614,7 +14614,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -14678,7 +14678,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -14742,7 +14742,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -14802,7 +14802,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -14866,7 +14866,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -14926,7 +14926,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВФУ</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -14986,7 +14986,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГУ</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -15050,7 +15050,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
@@ -15114,7 +15114,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БашГУ</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВятГУ</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -15242,7 +15242,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БашГУ</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -15306,7 +15306,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БайГУЭП</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВФУ</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -15430,7 +15430,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВолгГУ</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БрянГТУ</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -15686,7 +15686,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
@@ -15750,7 +15750,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
@@ -15814,7 +15814,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазГАСУ</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Сев(Аркт)ФУ</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
@@ -15942,7 +15942,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КургГУ</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КузГТУ</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВГТУ</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -16194,7 +16194,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
@@ -16258,7 +16258,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
@@ -16322,7 +16322,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -16386,7 +16386,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -16450,7 +16450,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -16514,7 +16514,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -16578,7 +16578,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВФУ</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -16642,7 +16642,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -16706,7 +16706,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
@@ -16770,7 +16770,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БрянГТУ</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
@@ -16834,7 +16834,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -16898,7 +16898,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -16962,7 +16962,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГВМетИ</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -17026,7 +17026,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -17090,7 +17090,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГЭУ</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -17150,7 +17150,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВятГУ</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -17214,7 +17214,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -17278,7 +17278,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КалмГУ</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
@@ -17342,7 +17342,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГГУ</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
@@ -17406,7 +17406,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -17470,7 +17470,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
@@ -17534,7 +17534,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -17598,7 +17598,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -17662,7 +17662,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтФУ</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
@@ -17726,7 +17726,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГТУ</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
@@ -17790,7 +17790,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БелГТхнУ</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -17854,7 +17854,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ЮЗГУ</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
@@ -17918,7 +17918,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -17982,7 +17982,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -18046,7 +18046,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -18106,7 +18106,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -18170,7 +18170,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -18234,7 +18234,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -18298,7 +18298,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БратГУ</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -18358,7 +18358,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КострГТУ</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -18422,7 +18422,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -18486,7 +18486,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БратГУ</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -18550,7 +18550,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГУ</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -18610,7 +18610,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КубГТхнУ</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -18674,7 +18674,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -18738,7 +18738,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИндУ</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -18802,7 +18802,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -18866,7 +18866,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГУПБио</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -18930,7 +18930,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГВМетИ</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -18994,7 +18994,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -19058,7 +19058,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДагГУ</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -19122,7 +19122,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -19186,7 +19186,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -19250,7 +19250,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИндУ</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -19310,7 +19310,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -19374,7 +19374,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -19434,7 +19434,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГЛТА</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -19498,7 +19498,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВСГУТиУ</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -19562,7 +19562,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -19626,7 +19626,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -19690,7 +19690,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтГТУ</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -19754,7 +19754,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ПовГТУ</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -19818,7 +19818,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -19882,7 +19882,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -19946,7 +19946,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВГТУ</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -20010,7 +20010,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -20074,7 +20074,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МагнГТУ</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -20138,7 +20138,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КузГТУ</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -20202,7 +20202,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БашГУ</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -20266,7 +20266,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИвГАСУ</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -20330,7 +20330,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -20394,7 +20394,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -20458,7 +20458,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -20522,7 +20522,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ПовГТУ</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -20586,7 +20586,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -20650,7 +20650,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -20714,7 +20714,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГТУ</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -20778,7 +20778,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -20842,7 +20842,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГУ</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -20906,7 +20906,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГУ</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -20970,7 +20970,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -21034,7 +21034,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГУПищП</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -21098,7 +21098,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -21150,7 +21150,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Сев(Аркт)ФУ</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -21202,7 +21202,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -21266,7 +21266,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КургГУ</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -21330,7 +21330,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КрГТУ</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -21394,7 +21394,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -21458,7 +21458,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СибФУ</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -21522,7 +21522,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>СКГГТхнА</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -21586,7 +21586,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -21650,7 +21650,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -21714,7 +21714,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ГУЦМиЗ</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -21778,7 +21778,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГУ</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -21842,7 +21842,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КузГТУ</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -21906,7 +21906,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГЛТА</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -21970,7 +21970,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -22034,7 +22034,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -22098,7 +22098,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУИТ</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
@@ -22162,7 +22162,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
@@ -22226,7 +22226,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИжГТУ</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -22290,7 +22290,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
@@ -22354,7 +22354,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГГУ</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -22418,7 +22418,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АмурГУ</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
@@ -22482,7 +22482,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КузГТУ</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
@@ -22546,7 +22546,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
@@ -22610,7 +22610,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
@@ -22674,7 +22674,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГУ</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
@@ -22738,7 +22738,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИЭМ</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -22802,7 +22802,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -22866,7 +22866,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -22930,7 +22930,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -22994,7 +22994,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГУНГ</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -23058,7 +23058,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГГУ</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -23122,7 +23122,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -23186,7 +23186,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
@@ -23250,7 +23250,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -23314,7 +23314,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -23378,7 +23378,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -23442,7 +23442,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -23506,7 +23506,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -23570,7 +23570,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -23634,7 +23634,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
@@ -23698,7 +23698,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
@@ -23762,7 +23762,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВолгГТУ</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
@@ -23826,7 +23826,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГТУ</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
@@ -23890,7 +23890,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ЛипГТУ</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
@@ -23954,7 +23954,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВятГУ</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
@@ -24010,7 +24010,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ИркГУ</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
@@ -24074,7 +24074,7 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДонГТУ</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
@@ -24138,7 +24138,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БрянГТУ</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
@@ -24202,7 +24202,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГИндУ</t>
         </is>
       </c>
       <c r="E376" t="inlineStr">
@@ -24266,7 +24266,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
@@ -24326,7 +24326,7 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ЮЗГУ</t>
         </is>
       </c>
       <c r="E378" t="inlineStr">
@@ -24390,7 +24390,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ДВГТУ</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
@@ -24454,7 +24454,7 @@
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E380" t="inlineStr">
@@ -24518,7 +24518,7 @@
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ГУЦМиЗ</t>
         </is>
       </c>
       <c r="E381" t="inlineStr">
@@ -24582,7 +24582,7 @@
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E382" t="inlineStr">
@@ -24646,7 +24646,7 @@
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E383" t="inlineStr">
@@ -24710,7 +24710,7 @@
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E384" t="inlineStr">
@@ -24774,7 +24774,7 @@
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГТекстУ</t>
         </is>
       </c>
       <c r="E385" t="inlineStr">
@@ -24838,7 +24838,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
@@ -24902,7 +24902,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -24966,7 +24966,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -25030,7 +25030,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
@@ -25094,7 +25094,7 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>РГГРУ</t>
         </is>
       </c>
       <c r="E390" t="inlineStr">
@@ -25158,7 +25158,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>АлтГТУ</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
@@ -25222,7 +25222,7 @@
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАИ</t>
         </is>
       </c>
       <c r="E392" t="inlineStr">
@@ -25286,7 +25286,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВладГУ</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
@@ -25350,7 +25350,7 @@
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
@@ -25402,7 +25402,7 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВолгГАСУ</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
@@ -25466,7 +25466,7 @@
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Каз(Прив)ФУ</t>
         </is>
       </c>
       <c r="E396" t="inlineStr">
@@ -25530,7 +25530,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МАТИ</t>
         </is>
       </c>
       <c r="E397" t="inlineStr">
@@ -25594,7 +25594,7 @@
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>ВорГУ</t>
         </is>
       </c>
       <c r="E398" t="inlineStr">
@@ -25658,7 +25658,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>КазНИТУ-КАИ</t>
         </is>
       </c>
       <c r="E399" t="inlineStr">
@@ -25722,7 +25722,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>МГТекстУ</t>
         </is>
       </c>
       <c r="E400" t="inlineStr">
@@ -25786,7 +25786,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>БалтГТУ</t>
         </is>
       </c>
       <c r="E401" t="inlineStr">

</xml_diff>